<commit_message>
Oatside May 2026: remove phantom trip 71-8009 28/05 (truck did not run)
GPS matched an ABNORMAL trip (Origin 02:47-06:27, Dest 20:04-21:37) but
the truck did not actually run per Oh. Removed via remove_matched_trips
+ exclude_50 override (blocks no_finish 100% since GPS still shows the
truck at origin that day).

Grand: 1,496,160 -> 1,485,120 (-11,040 = base 7,360 + one-trip 50% 3,680)
Verify: exports/06_Customer_Summary.csv; 71-8009 has no 28/05 row in
05_Trip_Detail.csv; unmatched legs unchanged (22).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Oatside/TransportRateCalculator/reports/oatside-apr2026/exports/00_Full_Workbook.xlsx
+++ b/Oatside/TransportRateCalculator/reports/oatside-apr2026/exports/00_Full_Workbook.xlsx
@@ -28,13 +28,13 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Customer_Summary'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Customer_Trips_Per_Day'!$A$1:$C$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Audit_Log'!$A$1:$J$124</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Trip_Detail'!$A$1:$Z$154</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Trips_Pricing_All'!$A$1:$G$154</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Trip_Detail'!$A$1:$Z$153</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Trips_Pricing_All'!$A$1:$G$153</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Unmatched_Log'!$A$1:$H$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Daily_Activity'!$A$1:$I$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Daily_Time_24h_Check'!$A$1:$M$121</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$124</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Daily_Time_24h_Check'!$A$1:$M$120</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$83</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Manual_Extra_Trips'!$A$1:$D$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Manual_Return_Trips'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'NoWork_Outbound_50pct'!$A$1:$G$1</definedName>
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09 15:05</t>
+          <t>2026-06-10 13:46</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>1121952</v>
+        <v>1114592</v>
       </c>
     </row>
     <row r="14">
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>337312</v>
+        <v>333632</v>
       </c>
     </row>
     <row r="21">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1496160</v>
+        <v>1485120</v>
       </c>
     </row>
   </sheetData>
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I124"/>
+  <dimension ref="A1:I123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4400,12 +4400,12 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D109" s="2" t="n">
@@ -4429,35 +4429,35 @@
     </row>
     <row r="110">
       <c r="A110" s="8" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D110" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E110" s="6" t="n">
         <v>7360</v>
       </c>
       <c r="F110" s="6" t="n">
-        <v>7360</v>
+        <v>14720</v>
       </c>
       <c r="G110" s="6" t="n">
-        <v>3680</v>
+        <v>0</v>
       </c>
       <c r="H110" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I110" s="6" t="n">
-        <v>11040</v>
+        <v>14720</v>
       </c>
     </row>
     <row r="111">
@@ -4466,7 +4466,7 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
@@ -4499,7 +4499,7 @@
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
@@ -4532,7 +4532,7 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
@@ -4565,64 +4565,64 @@
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D114" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E114" s="6" t="n">
         <v>7360</v>
       </c>
       <c r="F114" s="6" t="n">
-        <v>14720</v>
+        <v>7360</v>
       </c>
       <c r="G114" s="6" t="n">
-        <v>0</v>
+        <v>3680</v>
       </c>
       <c r="H114" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I114" s="6" t="n">
-        <v>14720</v>
+        <v>11040</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="9" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D115" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E115" s="7" t="n">
-        <v>7360</v>
+        <v>7264</v>
       </c>
       <c r="F115" s="7" t="n">
-        <v>7360</v>
+        <v>7264</v>
       </c>
       <c r="G115" s="7" t="n">
-        <v>3680</v>
+        <v>3632</v>
       </c>
       <c r="H115" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I115" s="7" t="n">
-        <v>11040</v>
+        <v>10896</v>
       </c>
     </row>
     <row r="116">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
@@ -4640,22 +4640,22 @@
         </is>
       </c>
       <c r="D116" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E116" s="6" t="n">
         <v>7264</v>
       </c>
       <c r="F116" s="6" t="n">
-        <v>7264</v>
+        <v>14528</v>
       </c>
       <c r="G116" s="6" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="H116" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I116" s="6" t="n">
-        <v>10896</v>
+        <v>14528</v>
       </c>
     </row>
     <row r="117">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
@@ -4673,22 +4673,22 @@
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E117" s="7" t="n">
         <v>7264</v>
       </c>
       <c r="F117" s="7" t="n">
-        <v>14528</v>
+        <v>7264</v>
       </c>
       <c r="G117" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="H117" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I117" s="7" t="n">
-        <v>14528</v>
+        <v>10896</v>
       </c>
     </row>
     <row r="118">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
@@ -4730,45 +4730,45 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E119" s="7" t="n">
         <v>7264</v>
       </c>
       <c r="F119" s="7" t="n">
-        <v>7264</v>
+        <v>14528</v>
       </c>
       <c r="G119" s="7" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="H119" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I119" s="7" t="n">
-        <v>10896</v>
+        <v>14528</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="8" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D120" s="5" t="n">
@@ -4796,7 +4796,7 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
@@ -4805,22 +4805,22 @@
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E121" s="7" t="n">
         <v>7264</v>
       </c>
       <c r="F121" s="7" t="n">
-        <v>14528</v>
+        <v>7264</v>
       </c>
       <c r="G121" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="H121" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I121" s="7" t="n">
-        <v>14528</v>
+        <v>10896</v>
       </c>
     </row>
     <row r="122">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
@@ -4862,12 +4862,12 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D123" s="2" t="n">
@@ -4889,41 +4889,8 @@
         <v>10896</v>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" s="8" t="n">
-        <v>46173</v>
-      </c>
-      <c r="B124" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C124" s="5" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D124" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E124" s="6" t="n">
-        <v>7264</v>
-      </c>
-      <c r="F124" s="6" t="n">
-        <v>7264</v>
-      </c>
-      <c r="G124" s="6" t="n">
-        <v>3632</v>
-      </c>
-      <c r="H124" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I124" s="6" t="n">
-        <v>10896</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I124"/>
+  <autoFilter ref="A1:I123"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4934,7 +4901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8127,12 +8094,12 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
@@ -8165,7 +8132,7 @@
     </row>
     <row r="77">
       <c r="A77" s="9" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
@@ -8194,7 +8161,7 @@
       <c r="H77" s="2" t="inlineStr"/>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr"/>
@@ -8207,16 +8174,16 @@
     </row>
     <row r="78">
       <c r="A78" s="8" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
@@ -8236,15 +8203,15 @@
       <c r="H78" s="5" t="inlineStr"/>
       <c r="I78" s="5" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="J78" s="5" t="inlineStr"/>
       <c r="K78" s="6" t="n">
-        <v>7360</v>
+        <v>7264</v>
       </c>
       <c r="L78" s="6" t="n">
-        <v>3680</v>
+        <v>3632</v>
       </c>
     </row>
     <row r="79">
@@ -8253,7 +8220,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -8295,7 +8262,7 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
@@ -8333,11 +8300,11 @@
     </row>
     <row r="81">
       <c r="A81" s="9" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -8362,7 +8329,7 @@
       <c r="H81" s="2" t="inlineStr"/>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr"/>
@@ -8379,7 +8346,7 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
@@ -8421,12 +8388,12 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -8457,50 +8424,8 @@
         <v>3632</v>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="8" t="n">
-        <v>46173</v>
-      </c>
-      <c r="B84" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C84" s="5" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D84" s="5" t="inlineStr">
-        <is>
-          <t>one_trip_billed_day</t>
-        </is>
-      </c>
-      <c r="E84" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F84" s="5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G84" s="5" t="inlineStr"/>
-      <c r="H84" s="5" t="inlineStr"/>
-      <c r="I84" s="5" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="J84" s="5" t="inlineStr"/>
-      <c r="K84" s="6" t="n">
-        <v>7264</v>
-      </c>
-      <c r="L84" s="6" t="n">
-        <v>3632</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L84"/>
+  <autoFilter ref="A1:L83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8967,7 +8892,7 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>1121952</v>
+        <v>1114592</v>
       </c>
     </row>
     <row r="3">
@@ -9027,7 +8952,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>337312</v>
+        <v>333632</v>
       </c>
     </row>
     <row r="7">
@@ -9057,7 +8982,7 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1496160</v>
+        <v>1485120</v>
       </c>
     </row>
   </sheetData>
@@ -9399,10 +9324,10 @@
         <v>46170</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
@@ -13598,26 +13523,26 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E109" s="7" t="n">
         <v>7360</v>
       </c>
       <c r="F109" s="7" t="n">
-        <v>7360</v>
+        <v>0</v>
       </c>
       <c r="G109" s="7" t="n">
-        <v>3680</v>
+        <v>0</v>
       </c>
       <c r="H109" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I109" s="7" t="n">
-        <v>11040</v>
+        <v>0</v>
       </c>
       <c r="J109" s="2" t="inlineStr">
         <is>
-          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว)</t>
+          <t>ไม่เก็บ [override: exclude_50] — รถไม่ได้วิ่งจริง — ตัดเที่ยวเดียวของวันออกจาก base แล้ว เหลือ 0 เที่ยว แต่ GPS เห็นรถที่โรงงาน → กัน no_finish 100% ลั่น (คู่กับ remove_matched_trips ใน oatside_config.json)</t>
         </is>
       </c>
     </row>
@@ -14203,7 +14128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z154"/>
+  <dimension ref="A1:Z153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25992,7 +25917,7 @@
     </row>
     <row r="134">
       <c r="A134" s="8" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B134" s="8" t="n">
         <v>46170</v>
@@ -26002,67 +25927,63 @@
       </c>
       <c r="D134" s="5" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="F134" s="5" t="inlineStr">
         <is>
-          <t>71-8009 ชรินทร์ หัวลาก10W</t>
+          <t>72-1217 เนื้อ หัวลาก10W ตระไคร้</t>
         </is>
       </c>
       <c r="G134" s="5" t="inlineStr">
         <is>
-          <t>5.24</t>
+          <t>2.38</t>
         </is>
       </c>
       <c r="H134" s="5" t="inlineStr">
         <is>
-          <t>5.24</t>
+          <t>2.37</t>
         </is>
       </c>
       <c r="I134" s="10" t="n">
-        <v>46170.11607638889</v>
+        <v>46170.58722222222</v>
       </c>
       <c r="J134" s="10" t="n">
-        <v>46170.26921296296</v>
+        <v>46170.89265046296</v>
       </c>
       <c r="K134" s="5" t="n">
-        <v>3.68</v>
+        <v>7.33</v>
       </c>
       <c r="L134" s="10" t="n">
-        <v>46170.83622685185</v>
+        <v>46170.96063657408</v>
       </c>
       <c r="M134" s="10" t="n">
-        <v>46170.9013425926</v>
+        <v>46171.30994212963</v>
       </c>
       <c r="N134" s="5" t="n">
-        <v>13.61</v>
+        <v>1.63</v>
       </c>
       <c r="O134" s="5" t="n">
-        <v>1.56</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="P134" s="5" t="n">
-        <v>1.56</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="Q134" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R134" s="5" t="n">
-        <v>18.85</v>
+        <v>17.35</v>
       </c>
       <c r="S134" s="5" t="n">
-        <v>18.85</v>
-      </c>
-      <c r="T134" s="5" t="inlineStr">
-        <is>
-          <t>ABNORMAL</t>
-        </is>
-      </c>
+        <v>17.35</v>
+      </c>
+      <c r="T134" s="5" t="n"/>
       <c r="U134" s="5" t="n">
         <v>1</v>
       </c>
@@ -26087,68 +26008,68 @@
         <v>46171</v>
       </c>
       <c r="B135" s="9" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="C135" s="9" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>72-1217 เนื้อ หัวลาก10W ตระไคร้</t>
+          <t>71-5042 ณัชพน หัวลาก10W</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>2.38</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
-          <t>2.37</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="I135" s="11" t="n">
-        <v>46170.58722222222</v>
+        <v>46171.16535879629</v>
       </c>
       <c r="J135" s="11" t="n">
-        <v>46170.89265046296</v>
+        <v>46171.27927083334</v>
       </c>
       <c r="K135" s="2" t="n">
-        <v>7.33</v>
+        <v>2.73</v>
       </c>
       <c r="L135" s="11" t="n">
-        <v>46170.96063657408</v>
+        <v>46171.37247685185</v>
       </c>
       <c r="M135" s="11" t="n">
-        <v>46171.30994212963</v>
+        <v>46171.61934027778</v>
       </c>
       <c r="N135" s="2" t="n">
-        <v>1.63</v>
+        <v>2.24</v>
       </c>
       <c r="O135" s="2" t="n">
-        <v>8.380000000000001</v>
+        <v>5.92</v>
       </c>
       <c r="P135" s="2" t="n">
-        <v>8.380000000000001</v>
+        <v>5.92</v>
       </c>
       <c r="Q135" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R135" s="2" t="n">
-        <v>17.35</v>
+        <v>10.9</v>
       </c>
       <c r="S135" s="2" t="n">
-        <v>17.35</v>
+        <v>10.9</v>
       </c>
       <c r="T135" s="2" t="n"/>
       <c r="U135" s="2" t="n">
@@ -26158,7 +26079,7 @@
         <v>7360</v>
       </c>
       <c r="W135" s="7" t="n">
-        <v>3680</v>
+        <v>0</v>
       </c>
       <c r="X135" s="7" t="n">
         <v>0</v>
@@ -26197,46 +26118,46 @@
       </c>
       <c r="G136" s="5" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="H136" s="5" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="I136" s="10" t="n">
-        <v>46171.16535879629</v>
+        <v>46171.78201388889</v>
       </c>
       <c r="J136" s="10" t="n">
-        <v>46171.27927083334</v>
+        <v>46171.89481481481</v>
       </c>
       <c r="K136" s="5" t="n">
-        <v>2.73</v>
+        <v>2.71</v>
       </c>
       <c r="L136" s="10" t="n">
-        <v>46171.37247685185</v>
+        <v>46171.96677083334</v>
       </c>
       <c r="M136" s="10" t="n">
-        <v>46171.61934027778</v>
+        <v>46172.09275462963</v>
       </c>
       <c r="N136" s="5" t="n">
-        <v>2.24</v>
+        <v>1.73</v>
       </c>
       <c r="O136" s="5" t="n">
-        <v>5.92</v>
+        <v>3.02</v>
       </c>
       <c r="P136" s="5" t="n">
-        <v>5.92</v>
+        <v>3.02</v>
       </c>
       <c r="Q136" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R136" s="5" t="n">
-        <v>10.9</v>
+        <v>7.46</v>
       </c>
       <c r="S136" s="5" t="n">
-        <v>10.9</v>
+        <v>7.46</v>
       </c>
       <c r="T136" s="5" t="n"/>
       <c r="U136" s="5" t="n">
@@ -26275,56 +26196,56 @@
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>71-5042 ณัชพน หัวลาก10W</t>
+          <t>71-8002 สมประสงค์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>7.25</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>8.28</t>
         </is>
       </c>
       <c r="I137" s="11" t="n">
-        <v>46171.78201388889</v>
+        <v>46171.33181712963</v>
       </c>
       <c r="J137" s="11" t="n">
-        <v>46171.89481481481</v>
+        <v>46171.60032407408</v>
       </c>
       <c r="K137" s="2" t="n">
-        <v>2.71</v>
+        <v>6.44</v>
       </c>
       <c r="L137" s="11" t="n">
-        <v>46171.96677083334</v>
+        <v>46171.67759259259</v>
       </c>
       <c r="M137" s="11" t="n">
-        <v>46172.09275462963</v>
+        <v>46171.70689814815</v>
       </c>
       <c r="N137" s="2" t="n">
-        <v>1.73</v>
+        <v>1.85</v>
       </c>
       <c r="O137" s="2" t="n">
-        <v>3.02</v>
+        <v>0.7</v>
       </c>
       <c r="P137" s="2" t="n">
-        <v>3.02</v>
+        <v>0.7</v>
       </c>
       <c r="Q137" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R137" s="2" t="n">
-        <v>7.46</v>
+        <v>9</v>
       </c>
       <c r="S137" s="2" t="n">
-        <v>7.46</v>
+        <v>9</v>
       </c>
       <c r="T137" s="2" t="n"/>
       <c r="U137" s="2" t="n">
@@ -26351,7 +26272,7 @@
         <v>46171</v>
       </c>
       <c r="B138" s="8" t="n">
-        <v>46171</v>
+        <v>46170</v>
       </c>
       <c r="C138" s="8" t="n">
         <v>46171</v>
@@ -26363,56 +26284,56 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="F138" s="5" t="inlineStr">
         <is>
-          <t>71-8002 สมประสงค์ หัวลาก10W</t>
+          <t>71-8003 โกสินทร์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G138" s="5" t="inlineStr">
         <is>
-          <t>7.25</t>
+          <t>10.4</t>
         </is>
       </c>
       <c r="H138" s="5" t="inlineStr">
         <is>
-          <t>8.28</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="I138" s="10" t="n">
-        <v>46171.33181712963</v>
+        <v>46170.99238425926</v>
       </c>
       <c r="J138" s="10" t="n">
-        <v>46171.60032407408</v>
+        <v>46171.28165509259</v>
       </c>
       <c r="K138" s="5" t="n">
-        <v>6.44</v>
+        <v>6.94</v>
       </c>
       <c r="L138" s="10" t="n">
-        <v>46171.67759259259</v>
+        <v>46171.3696875</v>
       </c>
       <c r="M138" s="10" t="n">
-        <v>46171.70689814815</v>
+        <v>46171.59075231481</v>
       </c>
       <c r="N138" s="5" t="n">
-        <v>1.85</v>
+        <v>2.11</v>
       </c>
       <c r="O138" s="5" t="n">
-        <v>0.7</v>
+        <v>5.31</v>
       </c>
       <c r="P138" s="5" t="n">
-        <v>0.7</v>
+        <v>5.31</v>
       </c>
       <c r="Q138" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R138" s="5" t="n">
-        <v>9</v>
+        <v>14.36</v>
       </c>
       <c r="S138" s="5" t="n">
-        <v>9</v>
+        <v>14.36</v>
       </c>
       <c r="T138" s="5" t="n"/>
       <c r="U138" s="5" t="n">
@@ -26439,7 +26360,7 @@
         <v>46171</v>
       </c>
       <c r="B139" s="9" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="C139" s="9" t="n">
         <v>46171</v>
@@ -26461,46 +26382,46 @@
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>10.5</t>
         </is>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="I139" s="11" t="n">
-        <v>46170.99238425926</v>
+        <v>46171.66229166667</v>
       </c>
       <c r="J139" s="11" t="n">
-        <v>46171.28165509259</v>
+        <v>46171.72710648148</v>
       </c>
       <c r="K139" s="2" t="n">
-        <v>6.94</v>
+        <v>1.56</v>
       </c>
       <c r="L139" s="11" t="n">
-        <v>46171.3696875</v>
+        <v>46171.82959490741</v>
       </c>
       <c r="M139" s="11" t="n">
-        <v>46171.59075231481</v>
+        <v>46171.94225694444</v>
       </c>
       <c r="N139" s="2" t="n">
-        <v>2.11</v>
+        <v>2.46</v>
       </c>
       <c r="O139" s="2" t="n">
-        <v>5.31</v>
+        <v>2.7</v>
       </c>
       <c r="P139" s="2" t="n">
-        <v>5.31</v>
+        <v>2.7</v>
       </c>
       <c r="Q139" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R139" s="2" t="n">
-        <v>14.36</v>
+        <v>6.72</v>
       </c>
       <c r="S139" s="2" t="n">
-        <v>14.36</v>
+        <v>6.72</v>
       </c>
       <c r="T139" s="2" t="n"/>
       <c r="U139" s="2" t="n">
@@ -26539,56 +26460,56 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="F140" s="5" t="inlineStr">
         <is>
-          <t>71-8003 โกสินทร์ หัวลาก10W</t>
+          <t>71-8009 ชรินทร์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G140" s="5" t="inlineStr">
         <is>
-          <t>10.5</t>
+          <t>5.25</t>
         </is>
       </c>
       <c r="H140" s="5" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>5.25</t>
         </is>
       </c>
       <c r="I140" s="10" t="n">
-        <v>46171.66229166667</v>
+        <v>46171.00243055556</v>
       </c>
       <c r="J140" s="10" t="n">
-        <v>46171.72710648148</v>
+        <v>46171.46831018518</v>
       </c>
       <c r="K140" s="5" t="n">
-        <v>1.56</v>
+        <v>11.18</v>
       </c>
       <c r="L140" s="10" t="n">
-        <v>46171.82959490741</v>
+        <v>46171.54582175926</v>
       </c>
       <c r="M140" s="10" t="n">
-        <v>46171.94225694444</v>
+        <v>46171.60834490741</v>
       </c>
       <c r="N140" s="5" t="n">
-        <v>2.46</v>
+        <v>1.86</v>
       </c>
       <c r="O140" s="5" t="n">
-        <v>2.7</v>
+        <v>1.5</v>
       </c>
       <c r="P140" s="5" t="n">
-        <v>2.7</v>
+        <v>1.5</v>
       </c>
       <c r="Q140" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R140" s="5" t="n">
-        <v>6.72</v>
+        <v>14.54</v>
       </c>
       <c r="S140" s="5" t="n">
-        <v>6.72</v>
+        <v>14.54</v>
       </c>
       <c r="T140" s="5" t="n"/>
       <c r="U140" s="5" t="n">
@@ -26637,46 +26558,46 @@
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>5.25</t>
+          <t>5.26</t>
         </is>
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
-          <t>5.25</t>
+          <t>5.26</t>
         </is>
       </c>
       <c r="I141" s="11" t="n">
-        <v>46171.00243055556</v>
+        <v>46171.67638888889</v>
       </c>
       <c r="J141" s="11" t="n">
-        <v>46171.46831018518</v>
+        <v>46171.7416087963</v>
       </c>
       <c r="K141" s="2" t="n">
-        <v>11.18</v>
+        <v>1.57</v>
       </c>
       <c r="L141" s="11" t="n">
-        <v>46171.54582175926</v>
+        <v>46171.82641203704</v>
       </c>
       <c r="M141" s="11" t="n">
-        <v>46171.60834490741</v>
+        <v>46171.875625</v>
       </c>
       <c r="N141" s="2" t="n">
-        <v>1.86</v>
+        <v>2.04</v>
       </c>
       <c r="O141" s="2" t="n">
-        <v>1.5</v>
+        <v>1.18</v>
       </c>
       <c r="P141" s="2" t="n">
-        <v>1.5</v>
+        <v>1.18</v>
       </c>
       <c r="Q141" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R141" s="2" t="n">
-        <v>14.54</v>
+        <v>4.78</v>
       </c>
       <c r="S141" s="2" t="n">
-        <v>14.54</v>
+        <v>4.78</v>
       </c>
       <c r="T141" s="2" t="n"/>
       <c r="U141" s="2" t="n">
@@ -26700,7 +26621,7 @@
     </row>
     <row r="142">
       <c r="A142" s="8" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B142" s="8" t="n">
         <v>46171</v>
@@ -26710,68 +26631,68 @@
       </c>
       <c r="D142" s="5" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="F142" s="5" t="inlineStr">
         <is>
-          <t>71-8009 ชรินทร์ หัวลาก10W</t>
+          <t>72-1217 เนื้อ หัวลาก10W ตระไคร้</t>
         </is>
       </c>
       <c r="G142" s="5" t="inlineStr">
         <is>
-          <t>5.26</t>
+          <t>2.39</t>
         </is>
       </c>
       <c r="H142" s="5" t="inlineStr">
         <is>
-          <t>5.26</t>
+          <t>2.38</t>
         </is>
       </c>
       <c r="I142" s="10" t="n">
-        <v>46171.67638888889</v>
+        <v>46171.72065972222</v>
       </c>
       <c r="J142" s="10" t="n">
-        <v>46171.7416087963</v>
+        <v>46171.87474537037</v>
       </c>
       <c r="K142" s="5" t="n">
-        <v>1.57</v>
+        <v>3.7</v>
       </c>
       <c r="L142" s="10" t="n">
-        <v>46171.82641203704</v>
+        <v>46171.94614583333</v>
       </c>
       <c r="M142" s="10" t="n">
-        <v>46171.875625</v>
+        <v>46172.63309027778</v>
       </c>
       <c r="N142" s="5" t="n">
-        <v>2.04</v>
+        <v>1.71</v>
       </c>
       <c r="O142" s="5" t="n">
-        <v>1.18</v>
+        <v>16.49</v>
       </c>
       <c r="P142" s="5" t="n">
-        <v>1.18</v>
+        <v>16.49</v>
       </c>
       <c r="Q142" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R142" s="5" t="n">
-        <v>4.78</v>
+        <v>21.9</v>
       </c>
       <c r="S142" s="5" t="n">
-        <v>4.78</v>
+        <v>21.9</v>
       </c>
       <c r="T142" s="5" t="n"/>
       <c r="U142" s="5" t="n">
         <v>1</v>
       </c>
       <c r="V142" s="6" t="n">
-        <v>7360</v>
+        <v>7264</v>
       </c>
       <c r="W142" s="6" t="n">
         <v>0</v>
@@ -26791,68 +26712,68 @@
         <v>46172</v>
       </c>
       <c r="B143" s="9" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="C143" s="9" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>72-1217 เนื้อ หัวลาก10W ตระไคร้</t>
+          <t>71-5042 ณัชพน หัวลาก10W</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>2.39</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
-          <t>2.38</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="I143" s="11" t="n">
-        <v>46171.72065972222</v>
+        <v>46172.32059027778</v>
       </c>
       <c r="J143" s="11" t="n">
-        <v>46171.87474537037</v>
+        <v>46172.47302083333</v>
       </c>
       <c r="K143" s="2" t="n">
-        <v>3.7</v>
+        <v>3.66</v>
       </c>
       <c r="L143" s="11" t="n">
-        <v>46171.94614583333</v>
+        <v>46172.56171296296</v>
       </c>
       <c r="M143" s="11" t="n">
-        <v>46172.63309027778</v>
+        <v>46172.81743055556</v>
       </c>
       <c r="N143" s="2" t="n">
-        <v>1.71</v>
+        <v>2.13</v>
       </c>
       <c r="O143" s="2" t="n">
-        <v>16.49</v>
+        <v>6.14</v>
       </c>
       <c r="P143" s="2" t="n">
-        <v>16.49</v>
+        <v>6.14</v>
       </c>
       <c r="Q143" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R143" s="2" t="n">
-        <v>21.9</v>
+        <v>11.92</v>
       </c>
       <c r="S143" s="2" t="n">
-        <v>21.9</v>
+        <v>11.92</v>
       </c>
       <c r="T143" s="2" t="n"/>
       <c r="U143" s="2" t="n">
@@ -26862,7 +26783,7 @@
         <v>7264</v>
       </c>
       <c r="W143" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="X143" s="7" t="n">
         <v>0</v>
@@ -26879,7 +26800,7 @@
         <v>46172</v>
       </c>
       <c r="B144" s="8" t="n">
-        <v>46172</v>
+        <v>46171</v>
       </c>
       <c r="C144" s="8" t="n">
         <v>46172</v>
@@ -26891,58 +26812,62 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="F144" s="5" t="inlineStr">
         <is>
-          <t>71-5042 ณัชพน หัวลาก10W</t>
+          <t>71-8002 สมประสงค์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G144" s="5" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>7.26</t>
         </is>
       </c>
       <c r="H144" s="5" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>8.29</t>
         </is>
       </c>
       <c r="I144" s="10" t="n">
-        <v>46172.32059027778</v>
+        <v>46171.82071759259</v>
       </c>
       <c r="J144" s="10" t="n">
-        <v>46172.47302083333</v>
+        <v>46171.92391203704</v>
       </c>
       <c r="K144" s="5" t="n">
-        <v>3.66</v>
+        <v>2.48</v>
       </c>
       <c r="L144" s="10" t="n">
-        <v>46172.56171296296</v>
+        <v>46172.29966435185</v>
       </c>
       <c r="M144" s="10" t="n">
-        <v>46172.81743055556</v>
+        <v>46172.37111111111</v>
       </c>
       <c r="N144" s="5" t="n">
-        <v>2.13</v>
+        <v>9.02</v>
       </c>
       <c r="O144" s="5" t="n">
-        <v>6.14</v>
+        <v>1.71</v>
       </c>
       <c r="P144" s="5" t="n">
-        <v>6.14</v>
+        <v>1.71</v>
       </c>
       <c r="Q144" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R144" s="5" t="n">
-        <v>11.92</v>
+        <v>13.21</v>
       </c>
       <c r="S144" s="5" t="n">
-        <v>11.92</v>
-      </c>
-      <c r="T144" s="5" t="n"/>
+        <v>13.21</v>
+      </c>
+      <c r="T144" s="5" t="inlineStr">
+        <is>
+          <t>ABNORMAL</t>
+        </is>
+      </c>
       <c r="U144" s="5" t="n">
         <v>1</v>
       </c>
@@ -26950,7 +26875,7 @@
         <v>7264</v>
       </c>
       <c r="W144" s="6" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="X144" s="6" t="n">
         <v>0</v>
@@ -26967,7 +26892,7 @@
         <v>46172</v>
       </c>
       <c r="B145" s="9" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="C145" s="9" t="n">
         <v>46172</v>
@@ -26989,52 +26914,48 @@
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>7.26</t>
+          <t>7.27</t>
         </is>
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
-          <t>8.29</t>
+          <t>8.30</t>
         </is>
       </c>
       <c r="I145" s="11" t="n">
-        <v>46171.82071759259</v>
+        <v>46172.43083333333</v>
       </c>
       <c r="J145" s="11" t="n">
-        <v>46171.92391203704</v>
+        <v>46172.52552083333</v>
       </c>
       <c r="K145" s="2" t="n">
-        <v>2.48</v>
+        <v>2.27</v>
       </c>
       <c r="L145" s="11" t="n">
-        <v>46172.29966435185</v>
+        <v>46172.61280092593</v>
       </c>
       <c r="M145" s="11" t="n">
-        <v>46172.37111111111</v>
+        <v>46172.86035879629</v>
       </c>
       <c r="N145" s="2" t="n">
-        <v>9.02</v>
+        <v>2.09</v>
       </c>
       <c r="O145" s="2" t="n">
-        <v>1.71</v>
+        <v>5.94</v>
       </c>
       <c r="P145" s="2" t="n">
-        <v>1.71</v>
+        <v>5.94</v>
       </c>
       <c r="Q145" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R145" s="2" t="n">
-        <v>13.21</v>
+        <v>10.31</v>
       </c>
       <c r="S145" s="2" t="n">
-        <v>13.21</v>
-      </c>
-      <c r="T145" s="2" t="inlineStr">
-        <is>
-          <t>ABNORMAL</t>
-        </is>
-      </c>
+        <v>10.31</v>
+      </c>
+      <c r="T145" s="2" t="n"/>
       <c r="U145" s="2" t="n">
         <v>1</v>
       </c>
@@ -27071,56 +26992,56 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="F146" s="5" t="inlineStr">
         <is>
-          <t>71-8002 สมประสงค์ หัวลาก10W</t>
+          <t>71-8003 โกสินทร์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G146" s="5" t="inlineStr">
         <is>
-          <t>7.27</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="H146" s="5" t="inlineStr">
         <is>
-          <t>8.30</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="I146" s="10" t="n">
-        <v>46172.43083333333</v>
+        <v>46172.03034722222</v>
       </c>
       <c r="J146" s="10" t="n">
-        <v>46172.52552083333</v>
+        <v>46172.28571759259</v>
       </c>
       <c r="K146" s="5" t="n">
-        <v>2.27</v>
+        <v>6.13</v>
       </c>
       <c r="L146" s="10" t="n">
-        <v>46172.61280092593</v>
+        <v>46172.36446759259</v>
       </c>
       <c r="M146" s="10" t="n">
-        <v>46172.86035879629</v>
+        <v>46172.49165509259</v>
       </c>
       <c r="N146" s="5" t="n">
-        <v>2.09</v>
+        <v>1.89</v>
       </c>
       <c r="O146" s="5" t="n">
-        <v>5.94</v>
+        <v>3.05</v>
       </c>
       <c r="P146" s="5" t="n">
-        <v>5.94</v>
+        <v>3.05</v>
       </c>
       <c r="Q146" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R146" s="5" t="n">
-        <v>10.31</v>
+        <v>11.07</v>
       </c>
       <c r="S146" s="5" t="n">
-        <v>10.31</v>
+        <v>11.07</v>
       </c>
       <c r="T146" s="5" t="n"/>
       <c r="U146" s="5" t="n">
@@ -27130,7 +27051,7 @@
         <v>7264</v>
       </c>
       <c r="W146" s="6" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="X146" s="6" t="n">
         <v>0</v>
@@ -27147,7 +27068,7 @@
         <v>46172</v>
       </c>
       <c r="B147" s="9" t="n">
-        <v>46172</v>
+        <v>46171</v>
       </c>
       <c r="C147" s="9" t="n">
         <v>46172</v>
@@ -27159,56 +27080,56 @@
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>71-8003 โกสินทร์ หัวลาก10W</t>
+          <t>71-8009 ชรินทร์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>5.27</t>
         </is>
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>5.27</t>
         </is>
       </c>
       <c r="I147" s="11" t="n">
-        <v>46172.03034722222</v>
+        <v>46171.99543981482</v>
       </c>
       <c r="J147" s="11" t="n">
-        <v>46172.28571759259</v>
+        <v>46172.2858449074</v>
       </c>
       <c r="K147" s="2" t="n">
-        <v>6.13</v>
+        <v>6.97</v>
       </c>
       <c r="L147" s="11" t="n">
-        <v>46172.36446759259</v>
+        <v>46172.40947916666</v>
       </c>
       <c r="M147" s="11" t="n">
-        <v>46172.49165509259</v>
+        <v>46172.62247685185</v>
       </c>
       <c r="N147" s="2" t="n">
-        <v>1.89</v>
+        <v>2.97</v>
       </c>
       <c r="O147" s="2" t="n">
-        <v>3.05</v>
+        <v>5.11</v>
       </c>
       <c r="P147" s="2" t="n">
-        <v>3.05</v>
+        <v>5.11</v>
       </c>
       <c r="Q147" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R147" s="2" t="n">
-        <v>11.07</v>
+        <v>15.05</v>
       </c>
       <c r="S147" s="2" t="n">
-        <v>11.07</v>
+        <v>15.05</v>
       </c>
       <c r="T147" s="2" t="n"/>
       <c r="U147" s="2" t="n">
@@ -27232,13 +27153,13 @@
     </row>
     <row r="148">
       <c r="A148" s="8" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B148" s="8" t="n">
         <v>46172</v>
       </c>
-      <c r="B148" s="8" t="n">
-        <v>46171</v>
-      </c>
       <c r="C148" s="8" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="D148" s="5" t="inlineStr">
         <is>
@@ -27247,56 +27168,56 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="F148" s="5" t="inlineStr">
         <is>
-          <t>71-8009 ชรินทร์ หัวลาก10W</t>
+          <t>71-5042 ณัชพน หัวลาก10W</t>
         </is>
       </c>
       <c r="G148" s="5" t="inlineStr">
         <is>
-          <t>5.27</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="H148" s="5" t="inlineStr">
         <is>
-          <t>5.27</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="I148" s="10" t="n">
-        <v>46171.99543981482</v>
+        <v>46172.945</v>
       </c>
       <c r="J148" s="10" t="n">
-        <v>46172.2858449074</v>
+        <v>46173.25171296296</v>
       </c>
       <c r="K148" s="5" t="n">
-        <v>6.97</v>
+        <v>7.36</v>
       </c>
       <c r="L148" s="10" t="n">
-        <v>46172.40947916666</v>
+        <v>46173.33864583333</v>
       </c>
       <c r="M148" s="10" t="n">
-        <v>46172.62247685185</v>
+        <v>46173.38333333333</v>
       </c>
       <c r="N148" s="5" t="n">
-        <v>2.97</v>
+        <v>2.09</v>
       </c>
       <c r="O148" s="5" t="n">
-        <v>5.11</v>
+        <v>1.07</v>
       </c>
       <c r="P148" s="5" t="n">
-        <v>5.11</v>
+        <v>1.07</v>
       </c>
       <c r="Q148" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R148" s="5" t="n">
-        <v>15.05</v>
+        <v>10.52</v>
       </c>
       <c r="S148" s="5" t="n">
-        <v>15.05</v>
+        <v>10.52</v>
       </c>
       <c r="T148" s="5" t="n"/>
       <c r="U148" s="5" t="n">
@@ -27306,7 +27227,7 @@
         <v>7264</v>
       </c>
       <c r="W148" s="6" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="X148" s="6" t="n">
         <v>0</v>
@@ -27323,7 +27244,7 @@
         <v>46173</v>
       </c>
       <c r="B149" s="9" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="C149" s="9" t="n">
         <v>46173</v>
@@ -27345,46 +27266,46 @@
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="I149" s="11" t="n">
-        <v>46172.945</v>
+        <v>46173.50255787037</v>
       </c>
       <c r="J149" s="11" t="n">
-        <v>46173.25171296296</v>
+        <v>46173.72892361111</v>
       </c>
       <c r="K149" s="2" t="n">
-        <v>7.36</v>
+        <v>5.43</v>
       </c>
       <c r="L149" s="11" t="n">
-        <v>46173.33864583333</v>
+        <v>46173.81170138889</v>
       </c>
       <c r="M149" s="11" t="n">
-        <v>46173.38333333333</v>
+        <v>46173.91047453704</v>
       </c>
       <c r="N149" s="2" t="n">
-        <v>2.09</v>
+        <v>1.99</v>
       </c>
       <c r="O149" s="2" t="n">
-        <v>1.07</v>
+        <v>2.37</v>
       </c>
       <c r="P149" s="2" t="n">
-        <v>1.07</v>
+        <v>2.37</v>
       </c>
       <c r="Q149" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R149" s="2" t="n">
-        <v>10.52</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="S149" s="2" t="n">
-        <v>10.52</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="T149" s="2" t="n"/>
       <c r="U149" s="2" t="n">
@@ -27411,7 +27332,7 @@
         <v>46173</v>
       </c>
       <c r="B150" s="8" t="n">
-        <v>46173</v>
+        <v>46172</v>
       </c>
       <c r="C150" s="8" t="n">
         <v>46173</v>
@@ -27423,56 +27344,56 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="F150" s="5" t="inlineStr">
         <is>
-          <t>71-5042 ณัชพน หัวลาก10W</t>
+          <t>71-8002 สมประสงค์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G150" s="5" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>7.28</t>
         </is>
       </c>
       <c r="H150" s="5" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>8.31</t>
         </is>
       </c>
       <c r="I150" s="10" t="n">
-        <v>46173.50255787037</v>
+        <v>46172.96576388889</v>
       </c>
       <c r="J150" s="10" t="n">
-        <v>46173.72892361111</v>
+        <v>46173.20033564815</v>
       </c>
       <c r="K150" s="5" t="n">
-        <v>5.43</v>
+        <v>5.63</v>
       </c>
       <c r="L150" s="10" t="n">
-        <v>46173.81170138889</v>
+        <v>46173.26480324074</v>
       </c>
       <c r="M150" s="10" t="n">
-        <v>46173.91047453704</v>
+        <v>46173.38116898148</v>
       </c>
       <c r="N150" s="5" t="n">
-        <v>1.99</v>
+        <v>1.55</v>
       </c>
       <c r="O150" s="5" t="n">
-        <v>2.37</v>
+        <v>2.79</v>
       </c>
       <c r="P150" s="5" t="n">
-        <v>2.37</v>
+        <v>2.79</v>
       </c>
       <c r="Q150" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R150" s="5" t="n">
-        <v>9.789999999999999</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="S150" s="5" t="n">
-        <v>9.789999999999999</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="T150" s="5" t="n"/>
       <c r="U150" s="5" t="n">
@@ -27482,7 +27403,7 @@
         <v>7264</v>
       </c>
       <c r="W150" s="6" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="X150" s="6" t="n">
         <v>0</v>
@@ -27511,56 +27432,56 @@
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>71-8002 สมประสงค์ หัวลาก10W</t>
+          <t>71-8009 ชรินทร์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>7.28</t>
+          <t>5.28</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
-          <t>8.31</t>
+          <t>5.28</t>
         </is>
       </c>
       <c r="I151" s="11" t="n">
-        <v>46172.96576388889</v>
+        <v>46172.97828703704</v>
       </c>
       <c r="J151" s="11" t="n">
-        <v>46173.20033564815</v>
+        <v>46173.5018287037</v>
       </c>
       <c r="K151" s="2" t="n">
-        <v>5.63</v>
+        <v>12.56</v>
       </c>
       <c r="L151" s="11" t="n">
-        <v>46173.26480324074</v>
+        <v>46173.57653935185</v>
       </c>
       <c r="M151" s="11" t="n">
-        <v>46173.38116898148</v>
+        <v>46173.62144675926</v>
       </c>
       <c r="N151" s="2" t="n">
-        <v>1.55</v>
+        <v>1.79</v>
       </c>
       <c r="O151" s="2" t="n">
-        <v>2.79</v>
+        <v>1.08</v>
       </c>
       <c r="P151" s="2" t="n">
-        <v>2.79</v>
+        <v>1.08</v>
       </c>
       <c r="Q151" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R151" s="2" t="n">
-        <v>9.970000000000001</v>
+        <v>15.44</v>
       </c>
       <c r="S151" s="2" t="n">
-        <v>9.970000000000001</v>
+        <v>15.44</v>
       </c>
       <c r="T151" s="2" t="n"/>
       <c r="U151" s="2" t="n">
@@ -27584,7 +27505,7 @@
     </row>
     <row r="152">
       <c r="A152" s="8" t="n">
-        <v>46173</v>
+        <v>46172</v>
       </c>
       <c r="B152" s="8" t="n">
         <v>46172</v>
@@ -27594,61 +27515,61 @@
       </c>
       <c r="D152" s="5" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="F152" s="5" t="inlineStr">
         <is>
-          <t>71-8009 ชรินทร์ หัวลาก10W</t>
+          <t>72-1217 เนื้อ หัวลาก10W ตระไคร้</t>
         </is>
       </c>
       <c r="G152" s="5" t="inlineStr">
         <is>
-          <t>5.28</t>
+          <t>2.40</t>
         </is>
       </c>
       <c r="H152" s="5" t="inlineStr">
         <is>
-          <t>5.28</t>
+          <t>2.39</t>
         </is>
       </c>
       <c r="I152" s="10" t="n">
-        <v>46172.97828703704</v>
+        <v>46172.75962962963</v>
       </c>
       <c r="J152" s="10" t="n">
-        <v>46173.5018287037</v>
+        <v>46173.02157407408</v>
       </c>
       <c r="K152" s="5" t="n">
-        <v>12.56</v>
+        <v>6.29</v>
       </c>
       <c r="L152" s="10" t="n">
-        <v>46173.57653935185</v>
+        <v>46173.09358796296</v>
       </c>
       <c r="M152" s="10" t="n">
-        <v>46173.62144675926</v>
+        <v>46173.18756944445</v>
       </c>
       <c r="N152" s="5" t="n">
-        <v>1.79</v>
+        <v>1.73</v>
       </c>
       <c r="O152" s="5" t="n">
-        <v>1.08</v>
+        <v>2.26</v>
       </c>
       <c r="P152" s="5" t="n">
-        <v>1.08</v>
+        <v>2.26</v>
       </c>
       <c r="Q152" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R152" s="5" t="n">
-        <v>15.44</v>
+        <v>10.27</v>
       </c>
       <c r="S152" s="5" t="n">
-        <v>15.44</v>
+        <v>10.27</v>
       </c>
       <c r="T152" s="5" t="n"/>
       <c r="U152" s="5" t="n">
@@ -27658,7 +27579,7 @@
         <v>7264</v>
       </c>
       <c r="W152" s="6" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="X152" s="6" t="n">
         <v>0</v>
@@ -27672,10 +27593,10 @@
     </row>
     <row r="153">
       <c r="A153" s="9" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="B153" s="9" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="C153" s="9" t="n">
         <v>46173</v>
@@ -27697,46 +27618,46 @@
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
+          <t>2.41</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
           <t>2.40</t>
         </is>
       </c>
-      <c r="H153" s="2" t="inlineStr">
-        <is>
-          <t>2.39</t>
-        </is>
-      </c>
       <c r="I153" s="11" t="n">
-        <v>46172.75962962963</v>
+        <v>46173.25349537037</v>
       </c>
       <c r="J153" s="11" t="n">
-        <v>46173.02157407408</v>
+        <v>46173.31078703704</v>
       </c>
       <c r="K153" s="2" t="n">
-        <v>6.29</v>
+        <v>1.38</v>
       </c>
       <c r="L153" s="11" t="n">
-        <v>46173.09358796296</v>
+        <v>46173.385625</v>
       </c>
       <c r="M153" s="11" t="n">
-        <v>46173.18756944445</v>
+        <v>46173.41065972222</v>
       </c>
       <c r="N153" s="2" t="n">
-        <v>1.73</v>
+        <v>1.8</v>
       </c>
       <c r="O153" s="2" t="n">
-        <v>2.26</v>
+        <v>0.6</v>
       </c>
       <c r="P153" s="2" t="n">
-        <v>2.26</v>
+        <v>0.6</v>
       </c>
       <c r="Q153" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R153" s="2" t="n">
-        <v>10.27</v>
+        <v>3.77</v>
       </c>
       <c r="S153" s="2" t="n">
-        <v>10.27</v>
+        <v>3.77</v>
       </c>
       <c r="T153" s="2" t="n"/>
       <c r="U153" s="2" t="n">
@@ -27746,7 +27667,7 @@
         <v>7264</v>
       </c>
       <c r="W153" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="X153" s="7" t="n">
         <v>0</v>
@@ -27758,96 +27679,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" s="8" t="n">
-        <v>46173</v>
-      </c>
-      <c r="B154" s="8" t="n">
-        <v>46173</v>
-      </c>
-      <c r="C154" s="8" t="n">
-        <v>46173</v>
-      </c>
-      <c r="D154" s="5" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="E154" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="F154" s="5" t="inlineStr">
-        <is>
-          <t>72-1217 เนื้อ หัวลาก10W ตระไคร้</t>
-        </is>
-      </c>
-      <c r="G154" s="5" t="inlineStr">
-        <is>
-          <t>2.41</t>
-        </is>
-      </c>
-      <c r="H154" s="5" t="inlineStr">
-        <is>
-          <t>2.40</t>
-        </is>
-      </c>
-      <c r="I154" s="10" t="n">
-        <v>46173.25349537037</v>
-      </c>
-      <c r="J154" s="10" t="n">
-        <v>46173.31078703704</v>
-      </c>
-      <c r="K154" s="5" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="L154" s="10" t="n">
-        <v>46173.385625</v>
-      </c>
-      <c r="M154" s="10" t="n">
-        <v>46173.41065972222</v>
-      </c>
-      <c r="N154" s="5" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="O154" s="5" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="P154" s="5" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="Q154" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R154" s="5" t="n">
-        <v>3.77</v>
-      </c>
-      <c r="S154" s="5" t="n">
-        <v>3.77</v>
-      </c>
-      <c r="T154" s="5" t="n"/>
-      <c r="U154" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="V154" s="6" t="n">
-        <v>7264</v>
-      </c>
-      <c r="W154" s="6" t="n">
-        <v>3632</v>
-      </c>
-      <c r="X154" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y154" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z154" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:Z154"/>
+  <autoFilter ref="A1:Z153"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -27858,7 +27691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G154"/>
+  <dimension ref="A1:G153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31213,7 +31046,7 @@
       </c>
       <c r="B134" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C134" s="6" t="n">
@@ -31234,18 +31067,18 @@
     </row>
     <row r="135">
       <c r="A135" s="9" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C135" s="7" t="n">
         <v>7360</v>
       </c>
       <c r="D135" s="7" t="n">
-        <v>3680</v>
+        <v>0</v>
       </c>
       <c r="E135" s="7" t="n">
         <v>0</v>
@@ -31288,7 +31121,7 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C137" s="7" t="n">
@@ -31313,7 +31146,7 @@
       </c>
       <c r="B138" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C138" s="6" t="n">
@@ -31363,7 +31196,7 @@
       </c>
       <c r="B140" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C140" s="6" t="n">
@@ -31413,11 +31246,11 @@
       </c>
       <c r="B142" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C142" s="6" t="n">
-        <v>7360</v>
+        <v>7264</v>
       </c>
       <c r="D142" s="6" t="n">
         <v>0</v>
@@ -31434,18 +31267,18 @@
     </row>
     <row r="143">
       <c r="A143" s="9" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C143" s="7" t="n">
         <v>7264</v>
       </c>
       <c r="D143" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="E143" s="7" t="n">
         <v>0</v>
@@ -31463,14 +31296,14 @@
       </c>
       <c r="B144" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C144" s="6" t="n">
         <v>7264</v>
       </c>
       <c r="D144" s="6" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="E144" s="6" t="n">
         <v>0</v>
@@ -31513,14 +31346,14 @@
       </c>
       <c r="B146" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C146" s="6" t="n">
         <v>7264</v>
       </c>
       <c r="D146" s="6" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="E146" s="6" t="n">
         <v>0</v>
@@ -31538,7 +31371,7 @@
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C147" s="7" t="n">
@@ -31559,18 +31392,18 @@
     </row>
     <row r="148">
       <c r="A148" s="8" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="B148" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C148" s="6" t="n">
         <v>7264</v>
       </c>
       <c r="D148" s="6" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="E148" s="6" t="n">
         <v>0</v>
@@ -31613,14 +31446,14 @@
       </c>
       <c r="B150" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C150" s="6" t="n">
         <v>7264</v>
       </c>
       <c r="D150" s="6" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="E150" s="6" t="n">
         <v>0</v>
@@ -31638,7 +31471,7 @@
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C151" s="7" t="n">
@@ -31663,14 +31496,14 @@
       </c>
       <c r="B152" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C152" s="6" t="n">
         <v>7264</v>
       </c>
       <c r="D152" s="6" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="E152" s="6" t="n">
         <v>0</v>
@@ -31695,7 +31528,7 @@
         <v>7264</v>
       </c>
       <c r="D153" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="E153" s="7" t="n">
         <v>0</v>
@@ -31707,33 +31540,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" s="8" t="n">
-        <v>46173</v>
-      </c>
-      <c r="B154" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C154" s="6" t="n">
-        <v>7264</v>
-      </c>
-      <c r="D154" s="6" t="n">
-        <v>3632</v>
-      </c>
-      <c r="E154" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F154" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G154" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G154"/>
+  <autoFilter ref="A1:G153"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -33364,22 +33172,22 @@
         <v>46170</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C29" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D29" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="D29" s="2" t="n">
-        <v>10</v>
-      </c>
       <c r="E29" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H29" s="2" t="n">
         <v>1</v>
@@ -33487,7 +33295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M121"/>
+  <dimension ref="A1:M120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -38421,25 +38229,25 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>18.85</v>
+        <v>16.5</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>3.68</v>
+        <v>3.28</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>1.56</v>
+        <v>11.61</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>13.61</v>
+        <v>1.61</v>
       </c>
       <c r="H105" s="2" t="n">
         <v>0</v>
@@ -38448,45 +38256,45 @@
         <v>0</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>3.68</v>
+        <v>3.28</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>1.56</v>
+        <v>11.61</v>
       </c>
       <c r="L105" s="2" t="n">
-        <v>18.85</v>
+        <v>16.5</v>
       </c>
       <c r="M105" s="2" t="n">
-        <v>5.15</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D106" s="5" t="n">
-        <v>16.5</v>
+        <v>18.35</v>
       </c>
       <c r="E106" s="5" t="n">
-        <v>3.28</v>
+        <v>5.44</v>
       </c>
       <c r="F106" s="5" t="n">
-        <v>11.61</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="G106" s="5" t="n">
-        <v>1.61</v>
+        <v>3.96</v>
       </c>
       <c r="H106" s="5" t="n">
         <v>0</v>
@@ -38495,16 +38303,16 @@
         <v>0</v>
       </c>
       <c r="J106" s="5" t="n">
-        <v>3.28</v>
+        <v>5.44</v>
       </c>
       <c r="K106" s="5" t="n">
-        <v>11.61</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="L106" s="5" t="n">
-        <v>16.5</v>
+        <v>18.35</v>
       </c>
       <c r="M106" s="5" t="n">
-        <v>7.5</v>
+        <v>5.65</v>
       </c>
     </row>
     <row r="107">
@@ -38515,7 +38323,7 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
@@ -38524,16 +38332,16 @@
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>18.35</v>
+        <v>18.22</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>5.44</v>
+        <v>7.66</v>
       </c>
       <c r="F107" s="2" t="n">
-        <v>8.949999999999999</v>
+        <v>7.12</v>
       </c>
       <c r="G107" s="2" t="n">
-        <v>3.96</v>
+        <v>3.44</v>
       </c>
       <c r="H107" s="2" t="n">
         <v>0</v>
@@ -38542,16 +38350,16 @@
         <v>0</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>5.44</v>
+        <v>7.66</v>
       </c>
       <c r="K107" s="2" t="n">
-        <v>8.949999999999999</v>
+        <v>7.12</v>
       </c>
       <c r="L107" s="2" t="n">
-        <v>18.35</v>
+        <v>18.22</v>
       </c>
       <c r="M107" s="2" t="n">
-        <v>5.65</v>
+        <v>5.78</v>
       </c>
     </row>
     <row r="108">
@@ -38562,7 +38370,7 @@
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
@@ -38571,16 +38379,16 @@
         </is>
       </c>
       <c r="D108" s="5" t="n">
-        <v>18.22</v>
+        <v>21.08</v>
       </c>
       <c r="E108" s="5" t="n">
-        <v>7.66</v>
+        <v>8.5</v>
       </c>
       <c r="F108" s="5" t="n">
-        <v>7.12</v>
+        <v>8.01</v>
       </c>
       <c r="G108" s="5" t="n">
-        <v>3.44</v>
+        <v>4.57</v>
       </c>
       <c r="H108" s="5" t="n">
         <v>0</v>
@@ -38589,16 +38397,16 @@
         <v>0</v>
       </c>
       <c r="J108" s="5" t="n">
-        <v>7.66</v>
+        <v>8.5</v>
       </c>
       <c r="K108" s="5" t="n">
-        <v>7.12</v>
+        <v>8.01</v>
       </c>
       <c r="L108" s="5" t="n">
-        <v>18.22</v>
+        <v>21.08</v>
       </c>
       <c r="M108" s="5" t="n">
-        <v>5.78</v>
+        <v>2.92</v>
       </c>
     </row>
     <row r="109">
@@ -38609,7 +38417,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -38618,16 +38426,16 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>21.08</v>
+        <v>19.32</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>8.5</v>
+        <v>12.75</v>
       </c>
       <c r="F109" s="2" t="n">
-        <v>8.01</v>
+        <v>2.68</v>
       </c>
       <c r="G109" s="2" t="n">
-        <v>4.57</v>
+        <v>3.9</v>
       </c>
       <c r="H109" s="2" t="n">
         <v>0</v>
@@ -38636,16 +38444,16 @@
         <v>0</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>8.5</v>
+        <v>12.75</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>8.01</v>
+        <v>2.68</v>
       </c>
       <c r="L109" s="2" t="n">
-        <v>21.08</v>
+        <v>19.32</v>
       </c>
       <c r="M109" s="2" t="n">
-        <v>2.92</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="110">
@@ -38656,25 +38464,25 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D110" s="5" t="n">
-        <v>19.32</v>
+        <v>17.35</v>
       </c>
       <c r="E110" s="5" t="n">
-        <v>12.75</v>
+        <v>7.33</v>
       </c>
       <c r="F110" s="5" t="n">
-        <v>2.68</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="G110" s="5" t="n">
-        <v>3.9</v>
+        <v>1.63</v>
       </c>
       <c r="H110" s="5" t="n">
         <v>0</v>
@@ -38683,45 +38491,45 @@
         <v>0</v>
       </c>
       <c r="J110" s="5" t="n">
-        <v>12.75</v>
+        <v>7.33</v>
       </c>
       <c r="K110" s="5" t="n">
-        <v>2.68</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="L110" s="5" t="n">
-        <v>19.32</v>
+        <v>17.35</v>
       </c>
       <c r="M110" s="5" t="n">
-        <v>4.68</v>
+        <v>6.65</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>17.35</v>
+        <v>11.92</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>7.33</v>
+        <v>3.66</v>
       </c>
       <c r="F111" s="2" t="n">
-        <v>8.380000000000001</v>
+        <v>6.14</v>
       </c>
       <c r="G111" s="2" t="n">
-        <v>1.63</v>
+        <v>2.13</v>
       </c>
       <c r="H111" s="2" t="n">
         <v>0</v>
@@ -38730,16 +38538,16 @@
         <v>0</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>7.33</v>
+        <v>3.66</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>8.380000000000001</v>
+        <v>6.14</v>
       </c>
       <c r="L111" s="2" t="n">
-        <v>17.35</v>
+        <v>11.92</v>
       </c>
       <c r="M111" s="2" t="n">
-        <v>6.65</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="112">
@@ -38750,7 +38558,7 @@
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
@@ -38759,16 +38567,16 @@
         </is>
       </c>
       <c r="D112" s="5" t="n">
-        <v>11.92</v>
+        <v>23.52</v>
       </c>
       <c r="E112" s="5" t="n">
-        <v>3.66</v>
+        <v>4.75</v>
       </c>
       <c r="F112" s="5" t="n">
-        <v>6.14</v>
+        <v>7.66</v>
       </c>
       <c r="G112" s="5" t="n">
-        <v>2.13</v>
+        <v>11.11</v>
       </c>
       <c r="H112" s="5" t="n">
         <v>0</v>
@@ -38777,16 +38585,16 @@
         <v>0</v>
       </c>
       <c r="J112" s="5" t="n">
-        <v>3.66</v>
+        <v>4.75</v>
       </c>
       <c r="K112" s="5" t="n">
-        <v>6.14</v>
+        <v>7.66</v>
       </c>
       <c r="L112" s="5" t="n">
-        <v>11.92</v>
+        <v>23.52</v>
       </c>
       <c r="M112" s="5" t="n">
-        <v>12.08</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="113">
@@ -38797,7 +38605,7 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
@@ -38806,34 +38614,34 @@
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>23.52</v>
+        <v>11.07</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>4.75</v>
+        <v>6.13</v>
       </c>
       <c r="F113" s="2" t="n">
-        <v>7.66</v>
+        <v>3.05</v>
       </c>
       <c r="G113" s="2" t="n">
-        <v>11.11</v>
+        <v>1.89</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>0</v>
+        <v>0.53</v>
       </c>
       <c r="I113" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>4.75</v>
+        <v>6.65</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>7.66</v>
+        <v>3.05</v>
       </c>
       <c r="L113" s="2" t="n">
-        <v>23.52</v>
+        <v>11.6</v>
       </c>
       <c r="M113" s="2" t="n">
-        <v>0.48</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="114">
@@ -38844,7 +38652,7 @@
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
@@ -38853,34 +38661,34 @@
         </is>
       </c>
       <c r="D114" s="5" t="n">
-        <v>11.07</v>
+        <v>15.05</v>
       </c>
       <c r="E114" s="5" t="n">
-        <v>6.13</v>
+        <v>6.97</v>
       </c>
       <c r="F114" s="5" t="n">
-        <v>3.05</v>
+        <v>5.11</v>
       </c>
       <c r="G114" s="5" t="n">
-        <v>1.89</v>
+        <v>2.97</v>
       </c>
       <c r="H114" s="5" t="n">
-        <v>0.53</v>
+        <v>0</v>
       </c>
       <c r="I114" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J114" s="5" t="n">
-        <v>6.65</v>
+        <v>6.97</v>
       </c>
       <c r="K114" s="5" t="n">
-        <v>3.05</v>
+        <v>5.11</v>
       </c>
       <c r="L114" s="5" t="n">
-        <v>11.6</v>
+        <v>15.05</v>
       </c>
       <c r="M114" s="5" t="n">
-        <v>12.4</v>
+        <v>8.949999999999999</v>
       </c>
     </row>
     <row r="115">
@@ -38891,25 +38699,25 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>15.05</v>
+        <v>32.17</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>6.97</v>
+        <v>9.98</v>
       </c>
       <c r="F115" s="2" t="n">
-        <v>5.11</v>
+        <v>18.74</v>
       </c>
       <c r="G115" s="2" t="n">
-        <v>2.97</v>
+        <v>3.44</v>
       </c>
       <c r="H115" s="2" t="n">
         <v>0</v>
@@ -38918,63 +38726,63 @@
         <v>0</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>6.97</v>
+        <v>9.98</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>5.11</v>
+        <v>18.74</v>
       </c>
       <c r="L115" s="2" t="n">
-        <v>15.05</v>
+        <v>32.17</v>
       </c>
       <c r="M115" s="2" t="n">
-        <v>8.949999999999999</v>
+        <v>-8.17</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D116" s="5" t="n">
-        <v>32.17</v>
+        <v>20.31</v>
       </c>
       <c r="E116" s="5" t="n">
-        <v>9.98</v>
+        <v>12.79</v>
       </c>
       <c r="F116" s="5" t="n">
-        <v>18.74</v>
+        <v>3.44</v>
       </c>
       <c r="G116" s="5" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="H116" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I116" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J116" s="5" t="n">
+        <v>12.79</v>
+      </c>
+      <c r="K116" s="5" t="n">
         <v>3.44</v>
       </c>
-      <c r="H116" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I116" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J116" s="5" t="n">
-        <v>9.98</v>
-      </c>
-      <c r="K116" s="5" t="n">
-        <v>18.74</v>
-      </c>
       <c r="L116" s="5" t="n">
-        <v>32.17</v>
+        <v>20.31</v>
       </c>
       <c r="M116" s="5" t="n">
-        <v>-8.17</v>
+        <v>3.69</v>
       </c>
     </row>
     <row r="117">
@@ -38985,7 +38793,7 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
@@ -38994,34 +38802,34 @@
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>20.31</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>12.79</v>
+        <v>5.63</v>
       </c>
       <c r="F117" s="2" t="n">
-        <v>3.44</v>
+        <v>2.79</v>
       </c>
       <c r="G117" s="2" t="n">
-        <v>4.07</v>
+        <v>1.55</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>0</v>
+        <v>13.11</v>
       </c>
       <c r="I117" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>12.79</v>
+        <v>18.73</v>
       </c>
       <c r="K117" s="2" t="n">
-        <v>3.44</v>
+        <v>2.79</v>
       </c>
       <c r="L117" s="2" t="n">
-        <v>20.31</v>
+        <v>23.07</v>
       </c>
       <c r="M117" s="2" t="n">
-        <v>3.69</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="118">
@@ -39032,7 +38840,7 @@
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
@@ -39041,34 +38849,34 @@
         </is>
       </c>
       <c r="D118" s="5" t="n">
-        <v>9.970000000000001</v>
+        <v>0</v>
       </c>
       <c r="E118" s="5" t="n">
-        <v>5.63</v>
+        <v>0</v>
       </c>
       <c r="F118" s="5" t="n">
-        <v>2.79</v>
+        <v>0</v>
       </c>
       <c r="G118" s="5" t="n">
-        <v>1.55</v>
+        <v>0</v>
       </c>
       <c r="H118" s="5" t="n">
-        <v>13.11</v>
+        <v>0.61</v>
       </c>
       <c r="I118" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J118" s="5" t="n">
-        <v>18.73</v>
+        <v>0.61</v>
       </c>
       <c r="K118" s="5" t="n">
-        <v>2.79</v>
+        <v>0</v>
       </c>
       <c r="L118" s="5" t="n">
-        <v>23.07</v>
+        <v>0.61</v>
       </c>
       <c r="M118" s="5" t="n">
-        <v>0.93</v>
+        <v>23.39</v>
       </c>
     </row>
     <row r="119">
@@ -39079,7 +38887,7 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
@@ -39088,34 +38896,34 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>0</v>
+        <v>15.44</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>0</v>
+        <v>12.56</v>
       </c>
       <c r="F119" s="2" t="n">
-        <v>0</v>
+        <v>1.08</v>
       </c>
       <c r="G119" s="2" t="n">
-        <v>0</v>
+        <v>1.79</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>0.61</v>
+        <v>0</v>
       </c>
       <c r="I119" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.61</v>
+        <v>12.56</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>0</v>
+        <v>1.08</v>
       </c>
       <c r="L119" s="2" t="n">
-        <v>0.61</v>
+        <v>15.44</v>
       </c>
       <c r="M119" s="2" t="n">
-        <v>23.39</v>
+        <v>8.56</v>
       </c>
     </row>
     <row r="120">
@@ -39126,94 +38934,47 @@
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D120" s="5" t="n">
-        <v>15.44</v>
+        <v>3.77</v>
       </c>
       <c r="E120" s="5" t="n">
-        <v>12.56</v>
+        <v>1.38</v>
       </c>
       <c r="F120" s="5" t="n">
-        <v>1.08</v>
+        <v>0.6</v>
       </c>
       <c r="G120" s="5" t="n">
-        <v>1.79</v>
+        <v>1.8</v>
       </c>
       <c r="H120" s="5" t="n">
-        <v>0</v>
+        <v>5.35</v>
       </c>
       <c r="I120" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J120" s="5" t="n">
-        <v>12.56</v>
+        <v>6.72</v>
       </c>
       <c r="K120" s="5" t="n">
-        <v>1.08</v>
+        <v>0.6</v>
       </c>
       <c r="L120" s="5" t="n">
-        <v>15.44</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="M120" s="5" t="n">
-        <v>8.56</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="B121" s="2" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C121" s="2" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D121" s="2" t="n">
-        <v>3.77</v>
-      </c>
-      <c r="E121" s="2" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="F121" s="2" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G121" s="2" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="H121" s="2" t="n">
-        <v>5.35</v>
-      </c>
-      <c r="I121" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J121" s="2" t="n">
-        <v>6.72</v>
-      </c>
-      <c r="K121" s="2" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="L121" s="2" t="n">
-        <v>9.119999999999999</v>
-      </c>
-      <c r="M121" s="2" t="n">
         <v>14.88</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M121"/>
+  <autoFilter ref="A1:M120"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>